<commit_message>
Reconciliacion de 12 documentos de producto/software, diagnostico de logica y vacios, y ajustes menores
- Agrega Arquitectura_Producto_Software/ (12 docs reconciliados con el resto del proyecto)
- Agrega 3 diagnosticos: completitud tecnica, elementos faltantes para operar, y logica/vacios post-reconciliacion
- Agrega datos de items transversales: azarosidad/control, biodata, reactivos alternativos (formato dual)
- Actualiza Fase2-11, matriz de scoring y banco de reactivos con los ajustes acumulados
- Actualiza DECISIONS.md, ASSUMPTIONS.md, PROGRESS.json con el historial de decisiones
- Ignora carpeta _to_delete/ (uso interno, no forma parte del proyecto)
</commit_message>
<xml_diff>
--- a/Fase6_Matriz_Scoring.xlsx
+++ b/Fase6_Matriz_Scoring.xlsx
@@ -11,7 +11,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pesos_Dimensiones" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen_Dimensiones" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Niveles_Corte" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notas" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEM_IC" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deseabilidad_Social" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Azarosidad_Control" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notas" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -65,12 +68,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -17482,8 +17488,8 @@
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -17525,12 +17531,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>[PENDIENTE DE DATO PILOTO]</t>
+          <t>0.0 [PROVISIONAL]</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>[PENDIENTE DE DATO PILOTO]</t>
+          <t>15.83 [PROVISIONAL]</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -17550,12 +17556,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>[PENDIENTE DE DATO PILOTO]</t>
+          <t>15.83 [PROVISIONAL]</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>[PENDIENTE DE DATO PILOTO]</t>
+          <t>31.67 [PROVISIONAL]</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -17575,12 +17581,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>[PENDIENTE DE DATO PILOTO]</t>
+          <t>31.67 [PROVISIONAL]</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>[PENDIENTE DE DATO PILOTO]</t>
+          <t>47.5 [PROVISIONAL]</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -17600,12 +17606,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>[PENDIENTE DE DATO PILOTO]</t>
+          <t>47.5 [PROVISIONAL]</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>[PENDIENTE DE DATO PILOTO]</t>
+          <t>63.33 [PROVISIONAL]</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -17625,12 +17631,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>[PENDIENTE DE DATO PILOTO]</t>
+          <t>63.33 [PROVISIONAL]</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>[PENDIENTE DE DATO PILOTO]</t>
+          <t>79.17 [PROVISIONAL]</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -17650,12 +17656,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>[PENDIENTE DE DATO PILOTO]</t>
+          <t>79.17 [PROVISIONAL]</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>[PENDIENTE DE DATO PILOTO]</t>
+          <t>95.0 [PROVISIONAL]</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -17664,14 +17670,17 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Los percentiles minimo/maximo de cada nivel NO se inventan (DECISIONS.md, 'Reglas de trabajo permanentes'): se completan con los percentiles reales de la muestra piloto (Fase 8-9). El IGI es 'mas alto = mejor' (DECISIONS.md punto 19): Nivel 1 = el IGI mas bajo (mayor riesgo), Nivel 6 = el IGI mas alto (mayor integridad). El semaforo (columna E) agrupa Nivel 1-2=Rojo, 3-4=Amarillo, 5-6=Verde (DECISIONS.md punto 22), y es independiente de la invalidacion: un resultado invalidado siempre se muestra en Gris sin importar su nivel (Fase 6 Modelo de Calculo, Seccion 10).</t>
+    <row r="9" ht="90" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>[2026-09-15] Los valores de las columnas C y D son PROVISIONALES: sextiles matematicos de la escala 0-95 del IGI (95/6 ~= 15.83 puntos por nivel), usados unicamente para tener un prototipo funcional mientras no exista muestra piloto - NO son percentiles reales de una poblacion y NO deben presentarse a ninguna persona ni empresa como una norma valida (DECISIONS.md, 'Reglas de trabajo permanentes': no inventar normas ficticias). En cuanto exista la muestra piloto (Fase 8-9), estos 12 valores se reemplazan por los percentiles reales calculados sobre esa muestra (Baremo General y, mas adelante, por pais - DECISIONS.md punto 39), y la etiqueta '[PROVISIONAL]' desaparece. El IGI es 'mas alto = mejor' (DECISIONS.md punto 19): Nivel 1 = el IGI mas bajo (mayor riesgo), Nivel 6 = el IGI mas alto (mayor integridad). El semaforo (columna E) agrupa Nivel 1-2=Rojo, 3-4=Amarillo, 5-6=Verde (DECISIONS.md punto 22), y es independiente de la invalidacion: un resultado invalidado siempre se muestra en Gris sin importar su nivel (Fase 6 Modelo de Calculo, Seccion 10).</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A9:E9"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17682,14 +17691,641 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="78" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Error estandar de medicion (SEM) e intervalo de confianza del 95% del IGI</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Valor / formula</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>IGI reportado (tomado de Resumen_Dimensiones, celda F24)</t>
+        </is>
+      </c>
+      <c r="B3">
+        <f>Resumen_Dimensiones!F24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Confiabilidad_IGI (Omega de McDonald sobre las dimensiones Nucleo; Alfa de Cronbach como referencia secundaria - DECISIONS.md punto 30)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>[PENDIENTE DE DATO PILOTO]</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>DesviacionEstandar_muestra_referencia (de la muestra piloto real, Fase 8-9)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>[PENDIENTE DE DATO PILOTO]</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>SEM = DesviacionEstandar_muestra_referencia x RAIZ(1 - Confiabilidad_IGI)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>[PENDIENTE DE DATO PILOTO]</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>IC_95% inferior = IGI_reportado - 1.96 x SEM</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>[PENDIENTE DE DATO PILOTO]</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>IC_95% superior = IGI_reportado + 1.96 x SEM</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>[PENDIENTE DE DATO PILOTO]</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Las celdas B5-B8 quedan en [PENDIENTE DE DATO PILOTO] porque Confiabilidad_IGI y DesviacionEstandar_muestra_referencia son datos empiricos que todavia no existen (dependen de la muestra piloto de la Fase 8-9), conforme a la regla ya vigente en DECISIONS.md de no inventar estadisticas reales (ver Fase 6 Modelo de Calculo, Seccion 9). Una vez exista el dato piloto, las celdas B5-B8 deben reemplazarse por formulas reales (B5 = B4*RAIZ(1-B3), B6 = B4-1.96*B5, B7 = B4+1.96*B5) y todo reporte (B2C y B2B) debe mostrar el IGI junto con este intervalo, no solo el numero puntual.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Escala de Deseabilidad Social - 5o indicador de validez del protocolo (NO entra al IGI ni a ninguna dimension)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>Pregunta (variante base)</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>Respuesta (0-4, editable, ejemplo)</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>Endosado (1 si Respuesta&gt;=3, es decir 'De acuerdo' o 'Totalmente de acuerdo')</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>DS01</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>¿Qué tan de acuerdo estás con la siguiente idea: "Nunca he sentido envidia de otra persona, ni siquiera un poco"?</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <f>IF(C4&gt;=3,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>DS02</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>¿Qué tan de acuerdo estás con la siguiente idea: "Jamás en mi vida he dicho una mentira, ni siquiera una mentira piadosa para no herir a alguien"?</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <f>IF(C5&gt;=3,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>DS03</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>¿Qué tan de acuerdo estás con la siguiente idea: "Siempre cumplo absolutamente todas mis promesas, sin ninguna excepción, sin importar las circunstancias"?</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6">
+        <f>IF(C6&gt;=3,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>DS04</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>¿Qué tan de acuerdo estás con la siguiente idea: "Nunca he tomado, ni una sola vez en mi vida, algo que no fuera mío, así fuera de mínimo valor"?</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7">
+        <f>IF(C7&gt;=3,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>DS05</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>¿Qué tan de acuerdo estás con la siguiente idea: "Jamás he sentido rabia o resentimiento hacia otra persona, sin importar lo que esa persona haya hecho"?</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8">
+        <f>IF(C8&gt;=3,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>DS06</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>¿Qué tan de acuerdo estás con la siguiente idea: "Nunca he criticado a otra persona a sus espaldas, ni una sola vez en mi vida"?</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9">
+        <f>IF(C9&gt;=3,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>DS07</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>¿Qué tan de acuerdo estás con la siguiente idea: "Siempre digo exactamente lo que pienso, sin filtrar nada, en cualquier situación, sin excepción"?</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10">
+        <f>IF(C10&gt;=3,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>DS08</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>¿Qué tan de acuerdo estás con la siguiente idea: "Jamás me he aprovechado de una situación, ni una sola vez, aunque nadie se fuera a enterar"?</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11">
+        <f>IF(C11&gt;=3,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Total de reactivos endosados ('De acuerdo'/'Totalmente de acuerdo')</t>
+        </is>
+      </c>
+      <c r="D12" s="3">
+        <f>SUM(D4:D11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Bandera de manejo de impresion (&gt;=6 de 8 =&gt; 'manejo de impresion alto')</t>
+        </is>
+      </c>
+      <c r="D13" s="3">
+        <f>IF(D12&gt;=6,"SI - manejo de impresion alto","No")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>6 o más de los 8 reactivos endosados en 'De acuerdo' o 'Totalmente de acuerdo' (valor 3 o 4) =&gt; manejo de impresión alto: el IGI se sigue calculando y mostrando con su valor real, en color gris, con advertencia visible (igual que los otros 4 indicadores, punto 23). Nunca se excluye ni se recalcula.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A15:D15"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Reactivos de control de Azarosidad - 1er indicador de validez del protocolo (NO entra al IGI ni a ninguna dimension)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>Mecanismo</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>Pregunta (variante base)</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>Opcion objetivo (unica correcta)</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>Respuesta marcada (editable, ejemplo)</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>Correcto (1 si coincide con el objetivo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>CTRL01</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>instrucción embebida</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Este reactivo es un control de atención, no evalúa tu opinión: para continuar, selecciona la opción "De acuerdo" en la escala que aparece a continuación.</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>De acuerdo</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>De acuerdo</t>
+        </is>
+      </c>
+      <c r="F4">
+        <f>IF(E4=D4,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>CTRL02</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>instrucción embebida</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Reactivo de control de atención: selecciona la opción "Rara vez" para confirmar que sigues leyendo cada pregunta con cuidado.</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Rara vez</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Rara vez</t>
+        </is>
+      </c>
+      <c r="F5">
+        <f>IF(E5=D5,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>CTRL03</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>instrucción embebida</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Este reactivo no describe una situación real: es un control de calidad de tus respuestas. Selecciona la opción "Poco probable".</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Poco probable</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Poco probable</t>
+        </is>
+      </c>
+      <c r="F6">
+        <f>IF(E6=D6,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>CTRL04</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>instrucción embebida</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Control de atención: para continuar, selecciona la opción "Ninguna vez" en la siguiente escala, sin importar tu historial real.</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Ninguna vez</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Ninguna vez</t>
+        </is>
+      </c>
+      <c r="F7">
+        <f>IF(E7=D7,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>CTRL05</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>trivia obvia</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>¿En qué continente se encuentra Ecuador?</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>América</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>América</t>
+        </is>
+      </c>
+      <c r="F8">
+        <f>IF(E8=D8,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>CTRL06</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>trivia obvia</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>¿De qué color es el cielo en un día despejado, sin nubes?</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Azul</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Azul</t>
+        </is>
+      </c>
+      <c r="F9">
+        <f>IF(E9=D9,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Total de reactivos de control fallados (de los aplicados en esta bateria)</t>
+        </is>
+      </c>
+      <c r="F10" s="3">
+        <f>COUNTIF(F4:F9,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Bandera de invalidacion por Azarosidad (1 fallo = alerta interna; 2 o mas = invalidacion total del protocolo)</t>
+        </is>
+      </c>
+      <c r="F11" s="3">
+        <f>IF(F10&gt;=2,"SI - invalidacion total",IF(F10=1,"Alerta interna (sin invalidar)","No"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="60" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Esta bateria de ejemplo precarga las 6 filas (CTRL01-CTRL06, columna 'Mecanismo' distingue instruccion embebida de trivia obvia); la cantidad real de controles a aplicar depende del tamano de la bateria (2 en B2C de 50 reactivos, 4 en baterias intermedias, 6 en la bateria completa de 210, siempre al menos 1 de cada mecanismo - ver azarosidad_control_data.json y Fase 2 Seccion 5.1bis). Fallar (no marcar la opción objetivo/correcta) 1 de los reactivos de control aplicados genera una alerta interna, sin invalidar el resultado. Fallar 2 o más se marca como invalidación total del protocolo (mismo tratamiento visual que los otros indicadores: el IGI y cada Puntaje_dimensión se siguen calculando y mostrando con su valor real, en color gris, con advertencia visible — Fase 6, Sección 11).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A13:F13"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>Fase 6 — Matriz de Scoring — Notas y convenciones (Version 4, 21 dimensiones x 10 reactivos)</t>
         </is>
@@ -17781,7 +18417,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>8. [DESCONOCIDO] Esta matriz no incorpora todavia los 4 indicadores de validez del protocolo (Azarosidad, Omision, Aquiescencia, Contradiccion, definidos en la Fase 2) como columnas de calculo automatico; se documentan en prosa en Fase6_Modelo_Calculo.docx y se ilustran manualmente en el ejemplo de la Fase 7. Automatizarlos como formulas de esta misma hoja es una mejora sugerida para una iteracion futura del archivo, una vez exista una interfaz real de aplicacion del test.</t>
+          <t>8. [DESCONOCIDO] Esta matriz no incorpora todavia los primeros 4 indicadores de validez del protocolo (Azarosidad, Omision, Aquiescencia, Contradiccion, definidos en la Fase 2) como columnas de calculo automatico; se documentan en prosa en Fase6_Modelo_Calculo.docx y se ilustran manualmente en el ejemplo de la Fase 7. Automatizarlos como formulas de esta misma hoja es una mejora sugerida para una iteracion futura del archivo, una vez exista una interfaz real de aplicacion del test.</t>
         </is>
       </c>
     </row>
@@ -17792,6 +18428,53 @@
       <c r="A21" t="inlineStr">
         <is>
           <t>9. [PENDIENTE] El multiplicador de nivel de exigencia por jerarquia de puesto (DECISIONS.md punto 27, que se aplica sobre el PRB antes de calcular el IGI) todavia no esta parametrizado como formula en esta hoja; su tabla completa de valores vive en CONFIDENCIAL_Formulas_Calculo_IGI.docx. Automatizarlo aqui (con un selector de nivel 1-6 y de 'tiene personal a cargo') queda como mejora pendiente para una proxima iteracion de este archivo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>10. [2026-09-11] Hoja 'SEM_IC' (DECISIONS.md punto 32, Fase 6 Modelo de Calculo Seccion 9): toma el IGI reportado directamente de 'Resumen_Dimensiones' y deja las celdas de Confiabilidad_IGI, DesviacionEstandar_muestra_referencia, SEM e IC_95% en [PENDIENTE DE DATO PILOTO] hasta que exista la muestra real de la Fase 8-9; las formulas ya estan documentadas en la propia hoja para completarlas ese dia sin rediseno.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>11. [2026-09-11] Hoja 'Deseabilidad_Social' (5o indicador de validez del protocolo, DECISIONS.md punto 35, Fase 12 Seccion 7): a diferencia de los reactivos de 'Reactivos', esta escala de 8 items NUNCA entra al PRB ni al IGI ni a ninguna Puntaje_dimension - es un indicador de validez independiente. La hoja ya automatiza el conteo de reactivos endosados y la bandera de 'manejo de impresion alto' (&gt;=6 de 8), que se muestra igual que los otros 4 indicadores (IGI en gris con advertencia, nunca excluido ni recalculado - Fase 6 Modelo de Calculo, Seccion 11.3).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>12. [2026-09-15] Hoja 'Niveles_Corte': las columnas Percentil_min/Percentil_max ya no estan en blanco - se completaron con sextiles PROVISIONALES de la escala 0-95 (95/6 ~= 15.83 por nivel), marcados explicitamente como '[PROVISIONAL]' en cada celda y en la nota de la fila 9. Esto permite operar un prototipo funcional (asignar un Nivel 1-6 a cualquier IGI calculado) sin esperar a la muestra piloto; en cuanto exista esa muestra (Fase 8-9), estos 12 valores se reemplazan por los percentiles reales y la etiqueta '[PROVISIONAL]' se retira (Fase 6 Modelo de Calculo, Seccion 10.1).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>13. [2026-09-15] Hoja 'Azarosidad_Control' (1er indicador de validez del protocolo, Fase 2 Seccion 5.1bis): 6 reactivos de control transversales (CTRL01-CTRL06) de 2 mecanismos distintos (CTRL01-04 instruccion embebida, CTRL05-06 trivia obvia de cultura general), cada uno con una unica opcion objetivo/correcta. Igual que 'Deseabilidad_Social', NUNCA entran al PRB ni al IGI ni a ninguna Puntaje_dimension. La hoja automatiza el conteo de fallos y la bandera de invalidacion (1 fallo = alerta interna; 2 o mas = invalidacion total del protocolo, mismo tratamiento visual que los otros 4 indicadores). La cantidad de controles realmente aplicados en una bateria concreta depende de su tamano (2 en B2C-50, 4 en baterias intermedias, 6 en la bateria completa de 210, siempre al menos 1 de cada mecanismo - ver azarosidad_control_data.json).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>14. [2026-09-15] Reactivos alternativos de opciones concretas (op1_alt/op2_alt/perc1_alt x 21 dimensiones, reactivos_alternativos_data.json) y bloque de bio-data (6 reactivos, biodata_data.json) documentados en Fase 2 Seccion 9; ninguno de los dos cambia esta matriz de scoring (los alternativos preservan el mismo indicador/direccion/par espejo que el reactivo clasico al que reemplazan opcionalmente, y la bio-data es puramente informativa, sin puntaje).</t>
         </is>
       </c>
     </row>

</xml_diff>